<commit_message>
Vista de cliente con sus casos en tarjetas, remisiones clicables y fila de clínica en la remisión
- Clientes: clic en un cliente abre sus casos en tarjetas con resumen (casos, remisiones, total)
  y en cada tarjeta las remisiones del caso; clic en cualquier parte de la fila abre la remisión
- Panel del caso: la fila completa de cada remisión abre la remisión
- Cuentas de cobro: clic en una remisión abre su detalle
- Remisión (Excel e impresión): fila nueva de Clínica, máximo 8 productos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/templates/remision.xlsx
+++ b/backend/templates/remision.xlsx
@@ -1,23 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EFA1C8-15D3-409A-AFCC-C472AB61997B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23256" windowHeight="12456" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="17" name="REMISION" state="visible" r:id="rId4"/>
+    <sheet name="REMISION" sheetId="17" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'REMISION'!$A$1:$E$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">REMISION!$A$1:$E$43</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Remision No</t>
   </si>
@@ -54,80 +68,84 @@
   <si>
     <t>RECIBI:</t>
   </si>
+  <si>
+    <t>Clinica :</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="_([$$-240A] * #,##0_);_([$$-240A] * (#,##0);_([$$-240A] * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot; #,##0"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot; #,##0_);[Red](&quot;$&quot; #,##0)"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00 [$€-1]_-;-* #,##0.00 [$€-1]_-;_-* &quot;-&quot;?? [$€-1]_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_([$$-240A]\ * #,##0_);_([$$-240A]\ * \(#,##0\);_([$$-240A]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;\ #,##0_);[Red]\(&quot;$&quot;\ #,##0\)"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="00000080"/>
-      <family val="1"/>
-      <sz val="18"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <color rgb="00000080"/>
-      <family val="1"/>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <color rgb="00000080"/>
+      <sz val="18"/>
+      <color rgb="FF000080"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="9"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color theme="1" tint="0.3499862666707358"/>
+      <sz val="14"/>
+      <color rgb="FF000080"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000080"/>
+      <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
+      <color theme="1" tint="0.34998626667073579"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
-      <color rgb="000000FF"/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="4" tint="-0.499984740745262"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="5">
@@ -139,7 +157,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -151,12 +169,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.5999938962981048"/>
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -169,14 +187,14 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top/>
       <bottom/>
@@ -185,19 +203,19 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom style="thin">
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </left>
       <right/>
       <top/>
@@ -206,14 +224,14 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </left>
       <right/>
       <top style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </bottom>
       <diagonal/>
     </border>
@@ -221,33 +239,33 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </left>
       <right/>
       <top style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -256,7 +274,7 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -264,78 +282,78 @@
     <border>
       <left/>
       <right style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top style="medium">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right/>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </right>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </right>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -344,64 +362,51 @@
         <color theme="0" tint="-0.249977111117893"/>
       </left>
       <right style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </right>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right/>
       <top style="thin">
         <color theme="0" tint="-0.249977111117893"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right style="thin">
-        <color rgb="00E3E3E3"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00C0C0C0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00C0C0C0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E3E3E3"/>
+        <color rgb="FFE3E3E3"/>
       </right>
       <top style="thin">
-        <color theme="0" tint="-0.1499984740745262"/>
+        <color theme="0" tint="-0.14999847407452621"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right/>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -411,13 +416,13 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="FFC0C0C0"/>
       </left>
       <right/>
       <top/>
@@ -428,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -439,44 +444,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -499,6 +474,123 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -511,125 +603,35 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -655,17 +657,17 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>174624</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>150812</xdr:rowOff>
+      <xdr:rowOff>23812</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>12700</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>152746</xdr:rowOff>
+      <xdr:rowOff>25746</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 1">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -684,8 +686,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
+          <a:off x="174624" y="646112"/>
+          <a:ext cx="7019926" cy="332134"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -697,22 +699,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>563563</xdr:colOff>
+      <xdr:colOff>569913</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>126999</xdr:rowOff>
+      <xdr:rowOff>69849</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2815912</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>50344</xdr:rowOff>
+      <xdr:colOff>2822262</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>285294</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -728,8 +730,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
+          <a:off x="1624013" y="69849"/>
+          <a:ext cx="2252349" cy="545645"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -753,10 +755,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 3">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -785,22 +787,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>603250</xdr:colOff>
+      <xdr:colOff>709476</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>430653</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>113152</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>252852</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 4">
+        <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -816,8 +818,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
+          <a:off x="893626" y="0"/>
+          <a:ext cx="591127" cy="583052"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -841,10 +843,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 5">
+        <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1219,41 +1221,40 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N39"/>
-  <sheetFormatPr defaultRowHeight="13.2" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.44140625" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="55.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7" max="8" width="11.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="43.44140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="20.88671875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="26.109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="11.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="55.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="1" customWidth="1"/>
+    <col min="7" max="8" width="11.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="43.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.85546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="26.140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
+    <row r="1" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="1"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="5"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -1266,469 +1267,407 @@
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
     </row>
-    <row r="3" ht="23.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="10"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="73"/>
       <c r="F3" s="3"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-    </row>
-    <row r="4" ht="13.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H3" s="8"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+    </row>
+    <row r="4" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="76"/>
       <c r="F4" s="3"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="12"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H4" s="10"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+    </row>
+    <row r="5" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="19"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="78"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="79"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
-      <c r="N5" s="12"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H5" s="11"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+    </row>
+    <row r="6" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="23"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="82"/>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H6" s="12"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="4"/>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="26"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="29"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H7" s="15"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+    </row>
+    <row r="8" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
       <c r="F8" s="3"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-    </row>
-    <row r="9" ht="12.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H8" s="15"/>
+      <c r="I8" s="19"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+    </row>
+    <row r="9" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="25" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
+      <c r="B9" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="18"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
       <c r="F9" s="3"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-    </row>
-    <row r="10" ht="12" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H9" s="15"/>
+      <c r="I9" s="19"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+    </row>
+    <row r="10" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="63"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="19"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+    </row>
+    <row r="11" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="30"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-    </row>
-    <row r="11" ht="12.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="25" t="s">
+      <c r="C11" s="63"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+    </row>
+    <row r="12" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="26"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-    </row>
-    <row r="12" ht="13.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="34" t="s">
+      <c r="C12" s="14"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+    </row>
+    <row r="13" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="4"/>
+      <c r="B13" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-    </row>
-    <row r="13" ht="13.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="3"/>
+      <c r="C13" s="66"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="67"/>
       <c r="G13" s="4"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H13" s="15"/>
+    </row>
+    <row r="14" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
-      <c r="B14" s="40" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="41" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="42"/>
-      <c r="E14" s="43" t="s">
-        <v>8</v>
-      </c>
+      <c r="B14" s="68"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
+      <c r="E14" s="70"/>
       <c r="F14" s="3"/>
       <c r="G14" s="4"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="44"/>
-      <c r="K14" s="45"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H14" s="16"/>
+    </row>
+    <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
-      <c r="B15" s="46"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="48">
-        <v>0</v>
-      </c>
-      <c r="E15" s="49">
-        <f>+B15*D15</f>
-        <v>0</v>
+      <c r="B15" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="24"/>
+      <c r="E15" s="25" t="s">
+        <v>8</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="51"/>
-      <c r="J15" s="52"/>
-      <c r="K15" s="53"/>
-    </row>
-    <row r="16" ht="13.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H15" s="26"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="27"/>
+    </row>
+    <row r="16" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="4"/>
-      <c r="B16" s="46"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="48">
-        <v>0</v>
-      </c>
-      <c r="E16" s="49">
-        <f>+B16*D16</f>
-        <v>0</v>
-      </c>
+      <c r="B16" s="28"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="31"/>
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
-      <c r="H16" s="44"/>
-      <c r="I16" s="51"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="55"/>
-    </row>
-    <row r="17" ht="13.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H16" s="32"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="34"/>
+      <c r="K16" s="35"/>
+    </row>
+    <row r="17" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4"/>
-      <c r="B17" s="46"/>
-      <c r="C17" s="54"/>
-      <c r="D17" s="56">
-        <v>0</v>
-      </c>
-      <c r="E17" s="57">
-        <f>+B17*D17</f>
-        <v>0</v>
-      </c>
+      <c r="B17" s="28"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="31"/>
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="51"/>
-      <c r="J17" s="52"/>
-      <c r="K17" s="55"/>
-    </row>
-    <row r="18" ht="14.25" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H17" s="26"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="36"/>
+    </row>
+    <row r="18" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4"/>
-      <c r="B18" s="46"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="56">
+      <c r="B18" s="28"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="37">
         <v>0</v>
       </c>
-      <c r="E18" s="57">
-        <f>+B18*D18</f>
+      <c r="E18" s="38">
+        <f t="shared" ref="E16:E23" si="0">+B18*D18</f>
         <v>0</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="51"/>
-      <c r="J18" s="58"/>
-      <c r="K18" s="55"/>
-    </row>
-    <row r="19" ht="14.25" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H18" s="26"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="36"/>
+    </row>
+    <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="59">
+      <c r="B19" s="28"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="37">
         <v>0</v>
       </c>
-      <c r="E19" s="57">
-        <f>+B19*D19</f>
+      <c r="E19" s="38">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F19" s="1"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="4"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="51"/>
-      <c r="J19" s="60"/>
-      <c r="K19" s="55"/>
-    </row>
-    <row r="20" ht="14.25" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H19" s="27"/>
+      <c r="I19" s="33"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="36"/>
+    </row>
+    <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="56">
+      <c r="B20" s="28"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="40">
         <v>0</v>
       </c>
-      <c r="E20" s="57">
-        <f>+B20*D20</f>
+      <c r="E20" s="38">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F20" s="1"/>
       <c r="G20" s="4"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="51"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="55"/>
-    </row>
-    <row r="21" ht="14.25" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H20" s="26"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="36"/>
+    </row>
+    <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4"/>
-      <c r="B21" s="62"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="48">
+      <c r="B21" s="28"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="37">
         <v>0</v>
       </c>
-      <c r="E21" s="57">
-        <f>+B21*D21</f>
+      <c r="E21" s="38">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F21" s="1"/>
       <c r="G21" s="4"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="64"/>
-      <c r="J21" s="58"/>
-      <c r="K21" s="55"/>
-    </row>
-    <row r="22" ht="14.25" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H21" s="27"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="39"/>
+      <c r="K21" s="36"/>
+    </row>
+    <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
-      <c r="B22" s="65"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="67">
+      <c r="B22" s="44"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="46">
         <v>0</v>
       </c>
-      <c r="E22" s="57">
-        <f>+B22*D22</f>
+      <c r="E22" s="38">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F22" s="1"/>
       <c r="G22" s="4"/>
-      <c r="H22" s="44"/>
-      <c r="I22" s="64"/>
-      <c r="J22" s="58"/>
-      <c r="K22" s="55"/>
-    </row>
-    <row r="23" ht="12.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H22" s="26"/>
+      <c r="I22" s="43"/>
+      <c r="J22" s="39"/>
+      <c r="K22" s="36"/>
+    </row>
+    <row r="23" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4"/>
-      <c r="B23" s="68"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="69">
+      <c r="B23" s="47"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="48">
         <v>0</v>
       </c>
-      <c r="E23" s="57">
-        <f>+B23*D23</f>
+      <c r="E23" s="38">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F23" s="70"/>
+      <c r="F23" s="49"/>
       <c r="G23" s="4"/>
-      <c r="H23" s="44"/>
-      <c r="I23" s="58"/>
-      <c r="J23" s="58"/>
-      <c r="K23" s="55"/>
-    </row>
-    <row r="24" ht="12.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H23" s="26"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="36"/>
+    </row>
+    <row r="24" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
-      <c r="B24" s="71"/>
-      <c r="C24" s="72"/>
-      <c r="D24" s="73" t="s">
+      <c r="B24" s="50"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="74">
-        <f>SUM(E15:E23)</f>
+      <c r="E24" s="53">
+        <f>SUM(E16:E23)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="70"/>
+      <c r="F24" s="49"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="75"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="75"/>
-      <c r="K24" s="55"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H24" s="54"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="54"/>
+      <c r="K24" s="36"/>
+    </row>
+    <row r="25" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="76" t="s">
+      <c r="C25" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="57"/>
       <c r="F25" s="3"/>
       <c r="G25" s="4"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="45"/>
-      <c r="J25" s="58"/>
-      <c r="K25" s="55"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="80"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="81"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="81"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="39"/>
+      <c r="K25" s="36"/>
+    </row>
+    <row r="26" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="C26" s="29"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="60"/>
+      <c r="G26" s="60"/>
+    </row>
+    <row r="27" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="C27" s="61"/>
+      <c r="D27" s="62"/>
+      <c r="E27" s="60"/>
+    </row>
+    <row r="28" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="81"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
+      <c r="E28" s="60"/>
+    </row>
+    <row r="29" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="D29" s="4"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
-    </row>
+    <row r="35" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="37" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="39" ht="12.75" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.35433070866141736" bottom="0" header="0" footer="0"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;8
-</oddFooter>
+    <oddFooter>&amp;C&amp;8</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>